<commit_message>
002 R1.3_3: larguero de 9.45 m del muro 1 en MCC10-14 (STD, Excel y DXF)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DbpSpoM7qi5cJ9LMKpwgVv
</commit_message>
<xml_diff>
--- a/002/002_AreasTributarias_NOSE_DOCK_H5_H6_R1.3_3.xlsx
+++ b/002/002_AreasTributarias_NOSE_DOCK_H5_H6_R1.3_3.xlsx
@@ -1207,7 +1207,7 @@
     <t xml:space="preserve">Franja superior de muros laterales que va a las vigas de alero</t>
   </si>
   <si>
-    <t xml:space="preserve">C. MURO FRONTAL — EJE 1 (Z = 0) — LARGUEROS MC4-14, MC10-12 Y MC10-14; DINTEL MCC10-14 (R1.3_3: LARGUEROS A 0.60 M, @1.20 M Y A 9.45 M)</t>
+    <t xml:space="preserve">C. MURO FRONTAL — EJE 1 (Z = 0) — LARGUEROS MC4-14, MC10-12 Y MC10-14; DINTEL Y LARGUERO DE 9.45 M MCC10-14 (R1.3_3: LARGUEROS A 0.60 M, @1.20 M Y A 9.45 M)</t>
   </si>
   <si>
     <t xml:space="preserve">Vanos: puerta de 1.22 × 2.40 m (X 0.60 a 1.82) con jambas HSS2 hasta el larguero de 3.00 m y dintel a 2.40 m; vano del nose dock de 5.10 × 6.60 m (X 2.32 a 7.42), sin carga. El dintel de la cortina va en la línea de 6.60 m. La franja de la base (0.00–0.30 m) baja directo a la cimentación.</t>
@@ -2068,10 +2068,10 @@
     <t xml:space="preserve">Largueros muros A/B claro 1-2 (0.60 a 7.80 m) y larguero 7.80 m del muro 1</t>
   </si>
   <si>
-    <t xml:space="preserve">Largueros muros A/B claro 2-3, 9.00 m claro 1-2 y 9.00/9.45 m del muro 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Largueros en cajón (9.45 m claro 1-2, 9.00 m claro 2-3) y dintel de 6.60 m</t>
+    <t xml:space="preserve">Largueros muros A/B claro 2-3, 9.00 m claro 1-2 y 9.00 m del muro 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remates de contraflambeos en cajón (9.45 m claro 1-2, 9.00 m claro 2-3 y 9.45 m del muro 1) y dintel de 6.60 m</t>
   </si>
   <si>
     <t xml:space="preserve">Largueros cortos del muro 1 y dintel de puerta</t>
@@ -12236,7 +12236,7 @@
         <v>9</v>
       </c>
       <c r="D95" s="8" t="s">
-        <v>462</v>
+        <v>448</v>
       </c>
       <c r="E95" s="23" t="n">
         <v>9.45</v>
@@ -16619,13 +16619,13 @@
         <v>462</v>
       </c>
       <c r="C32" s="7" t="n">
-        <v>124.16</v>
+        <v>114.08</v>
       </c>
       <c r="D32" s="33" t="n">
         <v>8.2789</v>
       </c>
       <c r="E32" s="19" t="n">
-        <v>805.198</v>
+        <v>739.831</v>
       </c>
       <c r="F32" s="10" t="s">
         <v>680</v>
@@ -16636,13 +16636,13 @@
         <v>448</v>
       </c>
       <c r="C33" s="7" t="n">
-        <v>42.08</v>
+        <v>52.16</v>
       </c>
       <c r="D33" s="33" t="n">
         <v>16.5577</v>
       </c>
       <c r="E33" s="19" t="n">
-        <v>545.791</v>
+        <v>676.532</v>
       </c>
       <c r="F33" s="10" t="s">
         <v>681</v>
@@ -16833,7 +16833,7 @@
       <c r="D41" s="8"/>
       <c r="E41" s="19" t="n">
         <f aca="false">SUM(E23:E40)</f>
-        <v>6880.449</v>
+        <v>6945.823</v>
       </c>
       <c r="F41" s="10" t="s">
         <v>696</v>
@@ -16874,7 +16874,7 @@
       </c>
       <c r="C45" s="11" t="n">
         <f aca="false">E41/1000</f>
-        <v>6.880449</v>
+        <v>6.945823</v>
       </c>
       <c r="D45" s="8" t="s">
         <v>699</v>
@@ -16964,7 +16964,7 @@
       </c>
       <c r="C50" s="11" t="n">
         <f aca="false">SUM(C45:C49)</f>
-        <v>12.607225878</v>
+        <v>12.672599878</v>
       </c>
       <c r="D50" s="8" t="s">
         <v>699</v>

</xml_diff>